<commit_message>
Refactor project into separate modules
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Half-Orc</t>
+          <t>Human</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1201,37 +1201,37 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="G2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H2" t="n">
         <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K2" t="n">
         <v>15</v>
       </c>
       <c r="L2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Finalize DnD character creator: inventory/abilities, tests, report, README
</commit_message>
<xml_diff>
--- a/game_data.xlsx
+++ b/game_data.xlsx
@@ -1104,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1183,6 +1183,16 @@
           <t>history</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>abilities</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1192,52 +1202,50 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Human</t>
+          <t>Half-Orc</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fighter</t>
+          <t>Wizard</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H2" t="n">
         <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="J2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K2" t="n">
         <v>15</v>
       </c>
       <c r="L2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="M2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N2" t="n">
-        <v>11</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>I was born in a small village near the forest border. From an early age, I was different from the others. While most children learned farming and trade, I spent my time exploring old ruins, listening to travelers, and dreaming of adventure. One day, after a mysterious fire destroyed part of my village, I decided to leave home and search for the truth behind what had happened. Since then, I have traveled across dangerous lands, gained new skills, and learned to survive on my own. My journey is not only about treasure or glory, but also about finding answers and discovering who I truly am.</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>